<commit_message>
JEV no fluxo diário: critério de impacto do JEV, regra de confiança 0,8, fila de revisão e classificação no site
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/validacao/jev_validacao_50.xlsx
+++ b/validacao/jev_validacao_50.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Classificar" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Regras" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legenda" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -64,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -76,6 +77,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -454,6 +456,7 @@
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="70" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,6 +510,11 @@
           <t>Comentário</t>
         </is>
       </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Por que o Claude sugeriu</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -537,10 +545,27 @@
           <t>Oferta Pública Secundária</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Oferta secundária: acionistas vendem ações; não entra nem sai caixa da empresa.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -571,10 +596,27 @@
           <t>Pricing Oferta Pública Secundária TRPL4</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Precificação da mesma oferta secundária do item 1.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -605,10 +647,27 @@
           <t>Vitória de Leilão para 5 Novos Projetos no Peru</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Leilão vencido: mais receita no futuro, mais capex e dívida antes. Saldo neutro para o credor atual.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -639,10 +698,27 @@
           <t>Reorganização Societária - Incorporação, Cisão ou Fusão da Companhia</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Reorganização societária muda a estrutura do devedor; impacto depende do detalhe, não do título.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -673,10 +749,27 @@
           <t>Vitoria do Lote 7 do Leilão de Transmissão Aneel 01/26 (2ªEtapa)</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Leilão vencido (mesma lógica do item 3).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -707,10 +800,27 @@
           <t>Proposta de Distribuição de Proventos</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Proventos são saída de caixa, mas proposta de rotina; mexe no caixa, por isso relevante.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -741,10 +851,27 @@
           <t>Conversão de Ações</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Conversão de ações entre classes: não afeta caixa nem dívida.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -775,10 +902,27 @@
           <t>Primeiro programa de recompra de ações da companhia</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Recompra de ações é remuneração ao acionista com caixa da empresa; pequena para o credor.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -809,10 +953,27 @@
           <t>Aquisição de lote no leilão ANEEL 02.2024</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Lote em leilão ANEEL (mesma lógica do item 3).</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -843,10 +1004,27 @@
           <t>TAESA celebra contrato para aquisição de 5 ativos de transmissão de energia</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Compra de 5 ativos: aumenta dívida e receita ao mesmo tempo.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -877,10 +1055,27 @@
           <t>Aquisição de ações de emissão da RIALMA IV</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Compra de participação em SPE (Rialma IV).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -911,10 +1106,27 @@
           <t>Celebração de acordo para a criação de plataforma de controle conjunto de ativos no Brasil entre La Caisse e Grupo Energía Bogotá</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Criação de controle conjunto (La Caisse + GEB) sobre os ativos: muda o controlador do grupo de risco.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -945,10 +1157,27 @@
           <t>Conclusão do descruzamento de participações na IE Madeira e IE Garanhuns</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Descruzamento de participações = troca de ativos entre sócios.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -979,10 +1208,27 @@
           <t>Conclusão da aquisição de Rialma IV</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Conclusão da compra do item 11.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1013,10 +1259,27 @@
           <t>Comunicado - Eleição Diretor Presidente</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Eleição de diretor: governança pura.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1047,10 +1310,27 @@
           <t>Apresentação de Resultados do 1T26</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de resultados; o título não diz se foram bons ou ruins.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1081,10 +1361,27 @@
           <t>Aviso ao Mercado - oferta pública de debênture -11ª emissão</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>nova_divida</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Aviso de oferta de nova debênture: mais dívida para financiar o plano, sem sinal de estresse.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1115,10 +1412,27 @@
           <t>Entrada em operação de Tangará</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>operacional</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Entrada em operação = começa a receber RAP do projeto.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1149,10 +1463,27 @@
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Título genérico; não dá para saber o assunto sem abrir o documento.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1183,10 +1514,27 @@
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Título genérico (mesmo caso do item 19).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1217,10 +1565,27 @@
           <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de resultados (como o item 16).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1251,10 +1616,27 @@
           <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Mudança em comitê de auditoria: governança pura.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1285,10 +1667,27 @@
           <t>Energização Jacarandá</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>operacional</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Energização de projeto = começa a receber RAP.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1319,10 +1718,27 @@
           <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de resultados (como o item 16).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1353,10 +1769,27 @@
           <t>Resgate Total Antecipado</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>pagamento_divida</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Resgate antecipado total: a série deixa de existir; neutro para os demais credores.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1387,10 +1820,27 @@
           <t>Aviso aos Debenturistas - Pgto de Juros 8a emissão</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>pagamento_divida</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Pagamento de juros de rotina.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1421,10 +1871,27 @@
           <t>Amortização||Liquidação||Pagamento de juros/remuneração</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>pagamento_divida</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Amortização e juros de rotina.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1455,10 +1922,27 @@
           <t>Pagamento de principal e juros da 1a Emissão de Debêntures Simples da IE Ivaí</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>pagamento_divida</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Pagamento de principal e juros de rotina (debênture da IE Ivaí).</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1489,10 +1973,27 @@
           <t>Amortização||Pagamento de juros/remuneração</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>pagamento_divida</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Amortização e juros de rotina.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1523,10 +2024,27 @@
           <t>Taesa (TAEE11) registra nova RAP de R$ 23 mi com SE Açailândia</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>operacional</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Nova RAP por reforço em subestação = receita adicional.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1557,10 +2075,27 @@
           <t>ISA Energia (ISAE3, ISAE4) anuncia potencial oferta de ações PN</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Oferta de ações preferenciais da própria empresa: entra capital próprio, ajuda a desalavancar.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1591,10 +2126,27 @@
           <t>ISA Energia (ISAE3, ISAE4) registra oferta de até 44,4 mi de ações PN</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Registro da mesma oferta do item 31.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1625,10 +2177,27 @@
           <t>ISA Energia (ISAE3) registra início da operação do projeto Jacarandá</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>operacional</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Início de operação do projeto Jacarandá (mesmo fato do item 23).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1659,10 +2228,27 @@
           <t>Alupar acelera ciclo de investimentos e projeta pico de alavancagem em 2028</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>negativo</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Projeção explícita de pico de alavancagem em 2028: mais risco para o credor no médio prazo.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1693,10 +2279,27 @@
           <t>Alupar (ALUP4) anuncia RAP de R$ 96,7 mi em leilão da Aneel</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr"/>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>RAP conquistada em leilão (mesmo fato do item 5).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1727,10 +2330,27 @@
           <t>JBS, BTG, Itaúsa, Taesa, Brava e mais ações para acompanhar hoje</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr"/>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Lista de várias empresas para acompanhar no dia: só cita a Taesa.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1761,10 +2381,27 @@
           <t>Taesa (TAEE11) anuncia renúncia de presidente do conselho</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr"/>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Renúncia de presidente do conselho: governança pura.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1795,10 +2432,27 @@
           <t>Alupar (ALUP11) 4T25: receita segue avançando, mas variações em custos mantêm margem estável; neutro.</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr"/>
-      <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Resultado do 4T25 com margem estável; a própria fonte classifica como neutro.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1829,10 +2483,27 @@
           <t>Taesa (TAEE11) conclui aquisição de ativos de transmissão por R$ 1,6 bi</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr"/>
-      <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="3" t="inlineStr"/>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Conclusão da compra do item 10.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1863,10 +2534,27 @@
           <t>Alupar capta R$ 2,45 bilhões em debêntures para financiar projetos de transmissão em SP, MG e GO</t>
         </is>
       </c>
-      <c r="G41" s="3" t="inlineStr"/>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>nova_divida</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Captação de R$ 2,45 bi para obras: mais dívida com destino definido; ver item 34 sobre alavancagem.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1897,10 +2585,27 @@
           <t>Phronesis atinge 5% das ações PN da Alupar (ALUP11)</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr"/>
-      <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>societario_governanca</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>Fundo passa a deter 5% das preferenciais: não muda controle nem caixa.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1931,10 +2636,27 @@
           <t>Taesa paga R$ 23 milhões em juros de debêntures e reforça previsibilidade no setor elétrico</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr"/>
-      <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="3" t="inlineStr"/>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>pagamento_divida</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>Pagamento de juros de rotina.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1965,10 +2687,27 @@
           <t>Taesa (TAEE11), Bradesco (BBDC4), Petrobras (PETR4) divulgam resultados do 2T23: veja agenda completa desta semana</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr"/>
-      <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="3" t="inlineStr"/>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>Agenda de resultados de várias empresas: só cita a Taesa.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -1999,10 +2738,27 @@
           <t>Análise - Debênture TPE - Renda Fixa - Transmissora Paraíso de Energia S.A. - SET/2028</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>Análise de crédito da própria debênture. Não há categoria para 'análise de crédito' na lista: ver nota na aba Regras.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2033,10 +2789,27 @@
           <t>Taesa (TAEE11): Resultados do 1T24</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr"/>
-      <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Resultados do 1T24; o título não diz a direção.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2067,10 +2840,27 @@
           <t>Análise - DEB EDP TRANSMISSAO SP-MG S/A - Renda Fixa - JUL/2039</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr"/>
-      <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>outro</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Análise de crédito da própria debênture (como o item 44).</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2101,10 +2891,27 @@
           <t>Taesa (TAEE11) capta R$ 1,3 bilhão com emissão de debêntures</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>nova_divida</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Captação de R$ 1,3 bi em debêntures.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2135,10 +2942,27 @@
           <t>ISA Energia (ISAE4) 1T26: Resultados Ajustados em Linha</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr"/>
-      <c r="H49" s="3" t="inlineStr"/>
-      <c r="I49" s="3" t="inlineStr"/>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Resultados ajustados em linha com o esperado.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2169,10 +2993,27 @@
           <t>Taesa (TAEE11): alavancagem está confortável, diz presidente da companhia após dados do 4T23</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr"/>
-      <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="3" t="inlineStr"/>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>positivo</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>Sinal explícito de alavancagem confortável dado pela empresa.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2203,10 +3044,27 @@
           <t>Alupar capta R$ 648,5 milhões com debêntures</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr"/>
-      <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr"/>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>nova_divida</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
       <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Captação de R$ 648,5 mi em debêntures (2019).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2282,6 +3140,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Descrição</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Como usar</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>As colunas amarelas já vêm com a sugestão do Claude. Revise linha a linha e troque o que discordar: a decisão final é sua. As sugestões foram feitas sem olhar as respostas do JEV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Ponto de vista</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Sempre o de quem detém debêntures do emissor (credor), não o do acionista.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Evento: nova_divida</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Captação de dívida (debêntures, empréstimos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Evento: pagamento_divida</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Juros, amortização ou resgate de dívida existente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Evento: aquisicao_venda</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Leilão vencido, compra ou venda de ativo/participação, troca de participações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Evento: operacional</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Energização, entrada em operação, licença, nova RAP por reforço.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Evento: societario_governanca</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Eleição/renúncia, comitês, reorganização, ofertas de ações, entrada de acionista, mudança de controle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Evento: resultado</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Resultados, guidance, proventos, recompra de ações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Evento: outro</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Título genérico ou lista de várias empresas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Impacto positivo</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Entra receita (nova operação ou RAP), cai dívida, entra capital próprio, ou sinal explícito de alavancagem confortável.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Impacto negativo</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Sinal explícito de mais risco: pico de alavancagem, inadimplência, rebaixamento, estresse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Impacto neutro</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>O resto, inclusive rotina de pagamento, nova dívida para obra e aquisições com receita associada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Trata do crédito? sim</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>O documento mexe com caixa, dívida, receita ou estrutura do emissor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Trata do crédito? não</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Governança pura, oferta em que só acionistas vendem, título genérico ou lista de empresas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Lacuna encontrada</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Itens 44 e 46 são análises de crédito da própria debênture e não cabem em nenhuma categoria; ficaram em 'outro'. Sugestão: criar a categoria 'analise_credito' na próxima versão.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>